<commit_message>
PAUSED: checkpoint, builds in flight
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017NMcBvUc2Vu9DKDdwmhqo4
</commit_message>
<xml_diff>
--- a/task197/golden/site_response_scorecard.xlsx
+++ b/task197/golden/site_response_scorecard.xlsx
@@ -25,7 +25,7 @@
     <numFmt numFmtId="164" formatCode="0.0#"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,6 +47,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="8"/>
     </font>
   </fonts>
   <fills count="3">
@@ -79,7 +83,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -90,6 +94,7 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1479,7 +1484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1698,6 +1703,13 @@
       </c>
       <c r="D15" t="n">
         <v>242.6</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Portfolio totals are rounded once from the unrounded period sums, per clause 5, so they need not equal the sum of the rounded rows above.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1711,7 +1723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="92" customWidth="1" min="1" max="1"/>
@@ -1820,39 +1832,53 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>delivery dates and rounded once. Episode counts are whole.</t>
+          <t>delivery dates and rounded once. A portfolio total is rounded once from the unrounded</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>period sums, so it need not equal the sum of the rounded rows it sits under. Episode</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>counts are whole.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>Meppelerdiep had no qualifying over-frequency episode in the window, so its</t>
         </is>
       </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>down-regulation gain is reported as none rather than as zero.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>down-regulation gain is reported as none rather than as zero.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>The Oosterhout metering point was replaced at the connection with effect from</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>2026-10-01; both codes are its own and both are included.</t>
         </is>

</xml_diff>